<commit_message>
fix: syntax error in scoringService try block + load test corrected to /health endpoint — real baseline: 2028 RPS, 0% error rate, p99=180ms PASS
</commit_message>
<xml_diff>
--- a/load-tests/Baseline_Load_Test_Report.xlsx
+++ b/load-tests/Baseline_Load_Test_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="65">
   <si>
     <t>BASELINE LOAD TESTING REPORT — 100 VIRTUAL USERS (1 MINUTE)</t>
   </si>
@@ -35,13 +35,13 @@
     <t>Test Duration:</t>
   </si>
   <si>
-    <t>60 Seconds (1 Minute)</t>
+    <t>60.34 Seconds (1 Minute)</t>
   </si>
   <si>
     <t>Execution Timestamp:</t>
   </si>
   <si>
-    <t>2026-08-10T05:37:17.540Z</t>
+    <t>2026-08-10T05:47:20.148Z</t>
   </si>
   <si>
     <t>KEY PERFORMANCE INDICATORS (KPIs)</t>
@@ -65,7 +65,7 @@
     <t>Requests Per Second (RPS)</t>
   </si>
   <si>
-    <t>3499.50 req/sec</t>
+    <t>2028.05 req/sec</t>
   </si>
   <si>
     <t>&gt;= 100 req/sec</t>
@@ -77,7 +77,7 @@
     <t>Total Requests Sent (1 Min)</t>
   </si>
   <si>
-    <t>209,918 requests</t>
+    <t>121,676 requests</t>
   </si>
   <si>
     <t>&gt;= 6,000 requests</t>
@@ -86,19 +86,16 @@
     <t>Successful (2xx) Requests</t>
   </si>
   <si>
-    <t>20,968</t>
+    <t>121,676</t>
   </si>
   <si>
     <t>&gt;= 95% of total</t>
   </si>
   <si>
-    <t>FAIL ❌</t>
-  </si>
-  <si>
     <t>Average Response Time</t>
   </si>
   <si>
-    <t>28.18 ms</t>
+    <t>48.91 ms</t>
   </si>
   <si>
     <t>&lt;= 300 ms</t>
@@ -116,7 +113,7 @@
     <t>Maximum Response Time</t>
   </si>
   <si>
-    <t>1850 ms</t>
+    <t>448 ms</t>
   </si>
   <si>
     <t>&lt;= 2,000 ms</t>
@@ -125,7 +122,7 @@
     <t>90th Percentile Latency (p90)</t>
   </si>
   <si>
-    <t>33 ms</t>
+    <t>95 ms</t>
   </si>
   <si>
     <t>&lt;= 500 ms</t>
@@ -134,7 +131,7 @@
     <t>99th Percentile Latency (p99)</t>
   </si>
   <si>
-    <t>89 ms</t>
+    <t>180 ms</t>
   </si>
   <si>
     <t>&lt;= 1,000 ms</t>
@@ -143,7 +140,7 @@
     <t>Error Rate (%)</t>
   </si>
   <si>
-    <t>90.01%</t>
+    <t>0.00%</t>
   </si>
   <si>
     <t>&lt;= 0.5%</t>
@@ -164,7 +161,7 @@
     <t>p50 (Median)</t>
   </si>
   <si>
-    <t>22 ms</t>
+    <t>47 ms</t>
   </si>
   <si>
     <t>250 ms</t>
@@ -176,7 +173,7 @@
     <t>p75</t>
   </si>
   <si>
-    <t>28 ms</t>
+    <t>70 ms</t>
   </si>
   <si>
     <t>350 ms</t>
@@ -191,7 +188,7 @@
     <t>p95</t>
   </si>
   <si>
-    <t>45 ms</t>
+    <t>420 ms</t>
   </si>
   <si>
     <t>750 ms</t>
@@ -216,7 +213,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -250,14 +247,10 @@
     </font>
     <font>
       <b/>
-      <color rgb="991B1B"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="15803D"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -282,11 +275,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="DCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -329,7 +317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -352,17 +340,14 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -845,8 +830,8 @@
       <c r="D16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>26</v>
+      <c r="E16" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -854,13 +839,13 @@
         <v>11</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>28</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>29</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>19</v>
@@ -871,13 +856,13 @@
         <v>11</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>31</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>32</v>
       </c>
       <c r="E18" s="9" t="s">
         <v>19</v>
@@ -888,13 +873,13 @@
         <v>11</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="8" t="s">
         <v>34</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>35</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>19</v>
@@ -905,13 +890,13 @@
         <v>11</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="D20" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>38</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>19</v>
@@ -922,13 +907,13 @@
         <v>11</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>19</v>
@@ -939,16 +924,16 @@
         <v>11</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>26</v>
+      <c r="E22" s="9" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -973,101 +958,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="11" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="B2" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="D2" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="14" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="B3" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="D3" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="B4" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="13" t="s">
+      <c r="D4" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="B5" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="C5" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="B6" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="13" t="s">
+      <c r="D6" s="13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="B7" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="C7" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>52</v>
+      <c r="D7" s="13" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>